<commit_message>
CONG THANH: use the user's corrected answer sheet as sample1 (100%)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_samples/CONG_THANH/sample1.xlsx
+++ b/test_samples/CONG_THANH/sample1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffrey.hu\Desktop\越南sample\VN-05 sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB07939-3918-4845-A6BF-5440E41135E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E4F22EF-B26C-4E40-9108-11E4C9B7A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="1110" windowWidth="34935" windowHeight="16680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="34935" windowHeight="16680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -582,31 +582,31 @@
     <xf numFmtId="179" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="5" fillId="0" borderId="6" xfId="6" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="5" fillId="0" borderId="7" xfId="7" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="5" fillId="0" borderId="7" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="179" fontId="5" fillId="0" borderId="7" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="16" fontId="5" fillId="0" borderId="6" xfId="6" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="5" fillId="0" borderId="7" xfId="7" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="5" fillId="0" borderId="7" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1522,30 +1522,30 @@
       <c r="I8" s="4"/>
     </row>
     <row r="9" spans="1:9" s="12" customFormat="1" ht="42" customHeight="1">
-      <c r="A9" s="42" t="s">
+      <c r="A9" s="44" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="42"/>
-      <c r="C9" s="42"/>
-      <c r="D9" s="42"/>
-      <c r="E9" s="42"/>
-      <c r="F9" s="42"/>
-      <c r="G9" s="42"/>
-      <c r="H9" s="42"/>
-      <c r="I9" s="42"/>
+      <c r="B9" s="44"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="44"/>
+      <c r="E9" s="44"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="44"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
     </row>
     <row r="10" spans="1:9" ht="22.5" customHeight="1" thickBot="1">
-      <c r="A10" s="43" t="s">
+      <c r="A10" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="43"/>
-      <c r="I10" s="43"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
+      <c r="D10" s="45"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="45"/>
+      <c r="G10" s="45"/>
+      <c r="H10" s="45"/>
+      <c r="I10" s="45"/>
     </row>
     <row r="11" spans="1:9" ht="36.75" customHeight="1" thickTop="1">
       <c r="A11" s="14" t="s">
@@ -1583,16 +1583,16 @@
       <c r="B12" s="41">
         <v>221014</v>
       </c>
-      <c r="C12" s="37" t="s">
+      <c r="C12" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="37">
+      <c r="D12" s="42">
         <v>1500000</v>
       </c>
-      <c r="E12" s="37">
+      <c r="E12" s="42">
         <v>120000</v>
       </c>
-      <c r="F12" s="37">
+      <c r="F12" s="42">
         <f>+D12+E12</f>
         <v>1620000</v>
       </c>
@@ -1602,94 +1602,94 @@
       <c r="H12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I12" s="38" t="s">
+      <c r="I12" s="43" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="12" customHeight="1">
       <c r="A13" s="39"/>
       <c r="B13" s="41"/>
-      <c r="C13" s="37" t="s">
+      <c r="C13" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="37"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="42"/>
       <c r="G13" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I13" s="38"/>
+      <c r="I13" s="43"/>
     </row>
     <row r="14" spans="1:9" ht="12" customHeight="1">
       <c r="A14" s="39"/>
       <c r="B14" s="41"/>
-      <c r="C14" s="37" t="s">
+      <c r="C14" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="37"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
       <c r="G14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I14" s="38"/>
+      <c r="I14" s="43"/>
     </row>
     <row r="15" spans="1:9" ht="12" customHeight="1">
       <c r="A15" s="39"/>
       <c r="B15" s="41"/>
-      <c r="C15" s="37" t="s">
+      <c r="C15" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="42"/>
+      <c r="F15" s="42"/>
       <c r="G15" s="1" t="s">
         <v>14</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I15" s="38"/>
+      <c r="I15" s="43"/>
     </row>
     <row r="16" spans="1:9" ht="12" customHeight="1">
       <c r="A16" s="39"/>
       <c r="B16" s="41"/>
-      <c r="C16" s="37" t="s">
+      <c r="C16" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="37"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="37"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="42"/>
       <c r="G16" s="1" t="s">
         <v>16</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="38"/>
+      <c r="I16" s="43"/>
     </row>
     <row r="17" spans="1:9" ht="12" customHeight="1">
       <c r="A17" s="39"/>
       <c r="B17" s="41"/>
-      <c r="C17" s="37" t="s">
+      <c r="C17" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="37"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="42"/>
+      <c r="F17" s="42"/>
       <c r="G17" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I17" s="38"/>
+      <c r="I17" s="43"/>
     </row>
     <row r="18" spans="1:9" ht="12" customHeight="1">
       <c r="A18" s="39">
@@ -1698,16 +1698,16 @@
       <c r="B18" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="37" t="s">
+      <c r="C18" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="37">
+      <c r="D18" s="42">
         <v>1824074</v>
       </c>
-      <c r="E18" s="37">
+      <c r="E18" s="42">
         <v>145926</v>
       </c>
-      <c r="F18" s="37">
+      <c r="F18" s="42">
         <f>+D18+E18</f>
         <v>1970000</v>
       </c>
@@ -1717,20 +1717,20 @@
       <c r="H18" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I18" s="38" t="s">
+      <c r="I18" s="43" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="12" customHeight="1">
       <c r="A19" s="39"/>
       <c r="B19" s="41"/>
-      <c r="C19" s="37" t="s">
+      <c r="C19" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="37">
-        <f t="shared" ref="F18:F23" si="0">+D19+E19</f>
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42">
+        <f t="shared" ref="F19:F23" si="0">+D19+E19</f>
         <v>0</v>
       </c>
       <c r="G19" s="1" t="s">
@@ -1739,17 +1739,17 @@
       <c r="H19" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I19" s="38"/>
+      <c r="I19" s="43"/>
     </row>
     <row r="20" spans="1:9" ht="12" customHeight="1">
       <c r="A20" s="39"/>
       <c r="B20" s="41"/>
-      <c r="C20" s="37" t="s">
+      <c r="C20" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="37"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="37">
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1759,17 +1759,17 @@
       <c r="H20" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I20" s="38"/>
+      <c r="I20" s="43"/>
     </row>
     <row r="21" spans="1:9" ht="12" customHeight="1">
       <c r="A21" s="39"/>
       <c r="B21" s="41"/>
-      <c r="C21" s="37" t="s">
+      <c r="C21" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="37"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="37">
+      <c r="D21" s="42"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1779,17 +1779,17 @@
       <c r="H21" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I21" s="38"/>
+      <c r="I21" s="43"/>
     </row>
     <row r="22" spans="1:9" ht="12" customHeight="1">
       <c r="A22" s="39"/>
       <c r="B22" s="41"/>
-      <c r="C22" s="37" t="s">
+      <c r="C22" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="37"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="37">
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1799,17 +1799,17 @@
       <c r="H22" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I22" s="38"/>
+      <c r="I22" s="43"/>
     </row>
     <row r="23" spans="1:9" ht="12" customHeight="1">
       <c r="A23" s="39"/>
       <c r="B23" s="41"/>
-      <c r="C23" s="37" t="s">
+      <c r="C23" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="37">
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+      <c r="F23" s="42">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1819,14 +1819,14 @@
       <c r="H23" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I23" s="38"/>
+      <c r="I23" s="43"/>
     </row>
     <row r="24" spans="1:9" s="22" customFormat="1" ht="12" customHeight="1" thickBot="1">
-      <c r="A24" s="44" t="s">
+      <c r="A24" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="45"/>
-      <c r="C24" s="45"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="38"/>
       <c r="D24" s="19">
         <f>SUM(D11:D23)</f>
         <v>3324074</v>
@@ -1891,11 +1891,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="A18:A23"/>
-    <mergeCell ref="B18:B23"/>
-    <mergeCell ref="C18:C23"/>
-    <mergeCell ref="D18:D23"/>
     <mergeCell ref="E18:E23"/>
     <mergeCell ref="F18:F23"/>
     <mergeCell ref="I18:I23"/>
@@ -1908,6 +1903,11 @@
     <mergeCell ref="E12:E17"/>
     <mergeCell ref="F12:F17"/>
     <mergeCell ref="I12:I17"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A18:A23"/>
+    <mergeCell ref="B18:B23"/>
+    <mergeCell ref="C18:C23"/>
+    <mergeCell ref="D18:D23"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <conditionalFormatting sqref="B1:B2 B4:B5">

</xml_diff>